<commit_message>
Correção dos Filtros de Modelo e Gestão, e correção da dinâmica dos filtros obrigatórios
</commit_message>
<xml_diff>
--- a/dimensoes.xlsx
+++ b/dimensoes.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PHONE STORE\Documents\PROJETIN_DOS_CRIA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D690D03-C434-4743-BA18-23A397D63979}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E5ACA27-4AEF-4755-86C6-066D5024BD1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{671B69D3-1FBE-4114-A181-B969F0E7BB39}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{671B69D3-1FBE-4114-A181-B969F0E7BB39}"/>
   </bookViews>
   <sheets>
     <sheet name="Lojas" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="693" uniqueCount="471">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="778" uniqueCount="525">
   <si>
     <t>V001</t>
   </si>
@@ -1450,13 +1450,175 @@
   </si>
   <si>
     <t>NOME PDV</t>
+  </si>
+  <si>
+    <t>PHONE STORE SHOP RIO ANIL SLZ</t>
+  </si>
+  <si>
+    <t>PHONE STORE IT CENTER</t>
+  </si>
+  <si>
+    <t>V207</t>
+  </si>
+  <si>
+    <t>EDUARDO MONTEIRO DE SOUZA (6)</t>
+  </si>
+  <si>
+    <t>V208</t>
+  </si>
+  <si>
+    <t>JHONATA TAVARES DOS SANTOS (452)</t>
+  </si>
+  <si>
+    <t>V209</t>
+  </si>
+  <si>
+    <t>JOÃO GABRIEL DO NASCIMENTO VILA NOVA (453)</t>
+  </si>
+  <si>
+    <t>V210</t>
+  </si>
+  <si>
+    <t>MARCOS VINICIUS OLIVEIRA DA SILVA (451)</t>
+  </si>
+  <si>
+    <t>V211</t>
+  </si>
+  <si>
+    <t>KAYKY PEREIRA PIRES (331)</t>
+  </si>
+  <si>
+    <t>V212</t>
+  </si>
+  <si>
+    <t>THAYRES SOUZA (424)</t>
+  </si>
+  <si>
+    <t>V213</t>
+  </si>
+  <si>
+    <t>JHULE MAIAN BARBOSA LOBATO (432)</t>
+  </si>
+  <si>
+    <t>V214</t>
+  </si>
+  <si>
+    <t>ANA.CLAUDIA.PHONESTORE (13)</t>
+  </si>
+  <si>
+    <t>V215</t>
+  </si>
+  <si>
+    <t>FERNANDO MATIAS DOS SANTOS MACHADO (455)</t>
+  </si>
+  <si>
+    <t>V216</t>
+  </si>
+  <si>
+    <t>FELIPE CAUÃ (454)</t>
+  </si>
+  <si>
+    <t>V217</t>
+  </si>
+  <si>
+    <t>JOAO GUSTAVO CARDOSO FERREIRA (456)</t>
+  </si>
+  <si>
+    <t>V218</t>
+  </si>
+  <si>
+    <t>MATEUS GABRIEL DE SOUSA VERA CRUZ (457)</t>
+  </si>
+  <si>
+    <t>V219</t>
+  </si>
+  <si>
+    <t>HARRISSON DE JESUS CALANDRINI CABRAL (459)</t>
+  </si>
+  <si>
+    <t>V220</t>
+  </si>
+  <si>
+    <t>JESSICA CRISTINA TORRES DOS SANTOS (458)</t>
+  </si>
+  <si>
+    <t>V221</t>
+  </si>
+  <si>
+    <t>LEONEL DE OLIVEIRA BARROS (461)</t>
+  </si>
+  <si>
+    <t>V222</t>
+  </si>
+  <si>
+    <t>ALESSANDRO GUIMARÃES LAMEIRA (460)</t>
+  </si>
+  <si>
+    <t>V223</t>
+  </si>
+  <si>
+    <t>BARBARA KAMILA SOUSA (463)</t>
+  </si>
+  <si>
+    <t>V224</t>
+  </si>
+  <si>
+    <t>MAYCON ROBERTH DE MELO BARROSO (462)</t>
+  </si>
+  <si>
+    <t>V225</t>
+  </si>
+  <si>
+    <t>THIAGO DOS SANTOS CHAVES (464)</t>
+  </si>
+  <si>
+    <t>V226</t>
+  </si>
+  <si>
+    <t>ELLEN CAROLINA CASTRO NASCIMENTO (465)</t>
+  </si>
+  <si>
+    <t>V227</t>
+  </si>
+  <si>
+    <t>LUCAS RAMON SOARES DO NASCIMENTO (58)</t>
+  </si>
+  <si>
+    <t>V228</t>
+  </si>
+  <si>
+    <t>ANDRIELY RAISSA DE CASTRO PALHETA (19)</t>
+  </si>
+  <si>
+    <t>V229</t>
+  </si>
+  <si>
+    <t>VICTOR SAMUEL CORRÊA GONÇALVES (467)</t>
+  </si>
+  <si>
+    <t>CLAUDIO RODRIGO COSTA SILVA (468)</t>
+  </si>
+  <si>
+    <t>V230</t>
+  </si>
+  <si>
+    <t>LUCAS TADEU OLIVEIRA DE AZEVEDO ( 8 )</t>
+  </si>
+  <si>
+    <t>LUCAS TADEU OLIVEIRA DE AZEVEDO (8)</t>
+  </si>
+  <si>
+    <t>V231</t>
+  </si>
+  <si>
+    <t>JOÃO FERNANDES SUP (13)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1472,8 +1634,15 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1490,6 +1659,12 @@
       <patternFill patternType="solid">
         <fgColor theme="1"/>
         <bgColor theme="1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD9D9D9"/>
+        <bgColor rgb="FFD9D9D9"/>
       </patternFill>
     </fill>
   </fills>
@@ -1542,7 +1717,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
@@ -1553,6 +1728,8 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1571,8 +1748,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C08398FD-EE49-41E3-99F2-04CCEA0E4D6A}" name="Tabela153" displayName="Tabela153" ref="A1:D22" totalsRowShown="0">
-  <autoFilter ref="A1:D22" xr:uid="{C08398FD-EE49-41E3-99F2-04CCEA0E4D6A}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C08398FD-EE49-41E3-99F2-04CCEA0E4D6A}" name="Tabela153" displayName="Tabela153" ref="A1:D24" totalsRowShown="0">
+  <autoFilter ref="A1:D24" xr:uid="{C08398FD-EE49-41E3-99F2-04CCEA0E4D6A}"/>
   <tableColumns count="4">
     <tableColumn id="7" xr3:uid="{C57A3094-E07F-4E89-94B2-73FC9F4A4EB5}" name="ID LOJA"/>
     <tableColumn id="8" xr3:uid="{99CA0D07-8487-4AE2-BE01-82406807DF39}" name="ID TIPO"/>
@@ -1891,7 +2068,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A165DF9A-B97A-4629-9B69-C646ABCECCBD}">
-  <dimension ref="A1:D22"/>
+  <dimension ref="A1:D24"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="4" width="28.109375" bestFit="1" customWidth="1"/>
@@ -2140,10 +2317,10 @@
         <v>17</v>
       </c>
       <c r="B18">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C18" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="D18" t="s">
         <v>430</v>
@@ -2203,6 +2380,34 @@
       </c>
       <c r="D22" t="s">
         <v>434</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A23">
+        <v>22</v>
+      </c>
+      <c r="B23">
+        <v>1</v>
+      </c>
+      <c r="C23" t="s">
+        <v>435</v>
+      </c>
+      <c r="D23" t="s">
+        <v>471</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A24">
+        <v>23</v>
+      </c>
+      <c r="B24">
+        <v>4</v>
+      </c>
+      <c r="C24" t="s">
+        <v>438</v>
+      </c>
+      <c r="D24" t="s">
+        <v>472</v>
       </c>
     </row>
   </sheetData>
@@ -2215,7 +2420,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F4489C6B-D1C2-415E-B0B3-CC749A9F03E5}">
-  <dimension ref="A1:C207"/>
+  <dimension ref="A1:C234"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.6640625" bestFit="1" customWidth="1"/>
@@ -4497,6 +4702,303 @@
         <v>413</v>
       </c>
       <c r="C207" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="208" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A208" s="1" t="s">
+        <v>473</v>
+      </c>
+      <c r="B208" s="2" t="s">
+        <v>474</v>
+      </c>
+      <c r="C208" s="3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="209" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A209" s="4" t="s">
+        <v>475</v>
+      </c>
+      <c r="B209" s="5" t="s">
+        <v>476</v>
+      </c>
+      <c r="C209" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="210" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A210" s="1" t="s">
+        <v>477</v>
+      </c>
+      <c r="B210" s="2" t="s">
+        <v>478</v>
+      </c>
+      <c r="C210" s="3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="211" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A211" s="4" t="s">
+        <v>479</v>
+      </c>
+      <c r="B211" s="5" t="s">
+        <v>480</v>
+      </c>
+      <c r="C211" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="212" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A212" s="1" t="s">
+        <v>481</v>
+      </c>
+      <c r="B212" s="2" t="s">
+        <v>482</v>
+      </c>
+      <c r="C212" s="3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="213" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A213" s="4" t="s">
+        <v>483</v>
+      </c>
+      <c r="B213" s="5" t="s">
+        <v>484</v>
+      </c>
+      <c r="C213" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="214" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A214" s="1" t="s">
+        <v>485</v>
+      </c>
+      <c r="B214" s="2" t="s">
+        <v>486</v>
+      </c>
+      <c r="C214" s="3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="215" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A215" s="4" t="s">
+        <v>487</v>
+      </c>
+      <c r="B215" s="5" t="s">
+        <v>488</v>
+      </c>
+      <c r="C215" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="216" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A216" s="1" t="s">
+        <v>489</v>
+      </c>
+      <c r="B216" s="2" t="s">
+        <v>490</v>
+      </c>
+      <c r="C216" s="3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="217" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A217" s="4" t="s">
+        <v>491</v>
+      </c>
+      <c r="B217" s="5" t="s">
+        <v>492</v>
+      </c>
+      <c r="C217" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="218" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A218" s="1" t="s">
+        <v>493</v>
+      </c>
+      <c r="B218" s="2" t="s">
+        <v>494</v>
+      </c>
+      <c r="C218" s="3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="219" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A219" s="4" t="s">
+        <v>495</v>
+      </c>
+      <c r="B219" s="5" t="s">
+        <v>496</v>
+      </c>
+      <c r="C219" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="220" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A220" s="1" t="s">
+        <v>497</v>
+      </c>
+      <c r="B220" s="2" t="s">
+        <v>498</v>
+      </c>
+      <c r="C220" s="3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="221" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A221" s="4" t="s">
+        <v>499</v>
+      </c>
+      <c r="B221" s="5" t="s">
+        <v>500</v>
+      </c>
+      <c r="C221" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="222" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A222" s="1" t="s">
+        <v>501</v>
+      </c>
+      <c r="B222" s="2" t="s">
+        <v>502</v>
+      </c>
+      <c r="C222" s="3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="223" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A223" s="4" t="s">
+        <v>503</v>
+      </c>
+      <c r="B223" s="5" t="s">
+        <v>504</v>
+      </c>
+      <c r="C223" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="224" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A224" s="1" t="s">
+        <v>505</v>
+      </c>
+      <c r="B224" s="10" t="s">
+        <v>506</v>
+      </c>
+      <c r="C224" s="3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="225" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A225" s="4" t="s">
+        <v>507</v>
+      </c>
+      <c r="B225" s="11" t="s">
+        <v>508</v>
+      </c>
+      <c r="C225" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="226" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A226" s="1" t="s">
+        <v>509</v>
+      </c>
+      <c r="B226" s="2" t="s">
+        <v>510</v>
+      </c>
+      <c r="C226" s="3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="227" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A227" s="4" t="s">
+        <v>511</v>
+      </c>
+      <c r="B227" s="5" t="s">
+        <v>512</v>
+      </c>
+      <c r="C227" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="228" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A228" s="1" t="s">
+        <v>513</v>
+      </c>
+      <c r="B228" s="10" t="s">
+        <v>514</v>
+      </c>
+      <c r="C228" s="3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="229" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A229" s="4" t="s">
+        <v>515</v>
+      </c>
+      <c r="B229" s="5" t="s">
+        <v>516</v>
+      </c>
+      <c r="C229" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="230" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A230" s="1" t="s">
+        <v>517</v>
+      </c>
+      <c r="B230" s="2" t="s">
+        <v>518</v>
+      </c>
+      <c r="C230" s="3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="231" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A231" s="4" t="s">
+        <v>517</v>
+      </c>
+      <c r="B231" s="5" t="s">
+        <v>519</v>
+      </c>
+      <c r="C231" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="232" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A232" s="1" t="s">
+        <v>520</v>
+      </c>
+      <c r="B232" s="2" t="s">
+        <v>521</v>
+      </c>
+      <c r="C232" s="3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="233" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A233" s="4" t="s">
+        <v>520</v>
+      </c>
+      <c r="B233" s="5" t="s">
+        <v>522</v>
+      </c>
+      <c r="C233" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="234" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A234" s="1" t="s">
+        <v>523</v>
+      </c>
+      <c r="B234" s="10" t="s">
+        <v>524</v>
+      </c>
+      <c r="C234" s="3" t="s">
         <v>17</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Implementação da visão de Vendedores 1.0
</commit_message>
<xml_diff>
--- a/dimensoes.xlsx
+++ b/dimensoes.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PHONE STORE\Documents\PROJETIN_DOS_CRIA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{692FBF60-3C77-4DF6-BE98-A3E910B08FD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1877B15D-FC1E-4AC3-8776-B74A6AF35D73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{671B69D3-1FBE-4114-A181-B969F0E7BB39}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{671B69D3-1FBE-4114-A181-B969F0E7BB39}"/>
   </bookViews>
   <sheets>
     <sheet name="Lojas" sheetId="1" r:id="rId1"/>
-    <sheet name="Vendedores" sheetId="2" r:id="rId2"/>
-    <sheet name="Planos" sheetId="3" r:id="rId3"/>
-    <sheet name="Categorias" sheetId="4" r:id="rId4"/>
+    <sheet name="Regiões" sheetId="5" r:id="rId2"/>
+    <sheet name="Vendedores" sheetId="2" r:id="rId3"/>
+    <sheet name="Planos" sheetId="3" r:id="rId4"/>
+    <sheet name="Categorias" sheetId="4" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="778" uniqueCount="525">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="851" uniqueCount="562">
   <si>
     <t>V001</t>
   </si>
@@ -1612,13 +1613,124 @@
   </si>
   <si>
     <t>PS - SHOP RIO ANIL SLZ</t>
+  </si>
+  <si>
+    <t>Rua Marly Sarney, 572- Centro, Açailândia - MA, 65930-000</t>
+  </si>
+  <si>
+    <t>AÇAILÂNIDA, MA</t>
+  </si>
+  <si>
+    <t>Rua Joao Alfredo 0239,Campina,Belém-PA,66013-000</t>
+  </si>
+  <si>
+    <t>BELÉM, PA</t>
+  </si>
+  <si>
+    <t>R. Boa Vista, 251 - Centro, Maceió - AL, 57020-110</t>
+  </si>
+  <si>
+    <t>MACEIÓ, AL</t>
+  </si>
+  <si>
+    <t>Av. Máximino Porpino da Silva, 1788 - Centro, Castanhal - PA, 68740-080</t>
+  </si>
+  <si>
+    <t>CASTANHAL, PA</t>
+  </si>
+  <si>
+    <t>Av. Dom Pedro II, 773-955 - Centro, Abaetetuba - PA, 68440-000</t>
+  </si>
+  <si>
+    <t>ABAETETUBA, PA</t>
+  </si>
+  <si>
+    <t>Av. Dom Pedro II, 24 - Centro, Abaetetuba - PA, 68440-000</t>
+  </si>
+  <si>
+    <t>Av. Barão do Rio Branco, 2480 - Centro, Castanhal - PA, 68743-050</t>
+  </si>
+  <si>
+    <t>Rodovia BR 316 km01, Castanheira, Belém - PA</t>
+  </si>
+  <si>
+    <t>Tv. SN 03, 753 - Cidade Nova, Ananindeua - PA, 67130-640</t>
+  </si>
+  <si>
+    <t>ANANINDEUA, PA</t>
+  </si>
+  <si>
+    <t>Rod. Mário Covas, 11590 - Coqueiro, Ananindeua - PA, 66650-000</t>
+  </si>
+  <si>
+    <t>Núcleo Residencial de Serviços - PA-275, Km 61 - 6 S/N, Parauapebas - PA, 68515-000</t>
+  </si>
+  <si>
+    <t>PARAUAPEBAS, RA</t>
+  </si>
+  <si>
+    <t>Tv. Padre Eutíquio, 1078 - Batista Campos, Belém - PA, 66023-710</t>
+  </si>
+  <si>
+    <t>Terminal Rodoviário de Belem - São Brás, Belém - PA, 66090-500</t>
+  </si>
+  <si>
+    <t>PS -  CAUCAIA</t>
+  </si>
+  <si>
+    <t>Avenida Edson da Mota Correia, 620</t>
+  </si>
+  <si>
+    <t>CAUCAIA, CE</t>
+  </si>
+  <si>
+    <t>PORTO VELHO, RO</t>
+  </si>
+  <si>
+    <t>MACAPÁ, AP</t>
+  </si>
+  <si>
+    <t>CAPANEMA, PA</t>
+  </si>
+  <si>
+    <t>ICOARACI, PA</t>
+  </si>
+  <si>
+    <t>PDV</t>
+  </si>
+  <si>
+    <t>ENDERECO</t>
+  </si>
+  <si>
+    <t>LOCALIZAÇÃO</t>
+  </si>
+  <si>
+    <t>Av. São Luís Rei de França, 8 - Turu, São Luís - MA, 65065-470</t>
+  </si>
+  <si>
+    <t>SÃO LUÍS, MA</t>
+  </si>
+  <si>
+    <t>Av. Prefeito Chiquilito Erse, 3288, Flodoaldo Pontes Pinto, Porto Velho - RO,76820-408</t>
+  </si>
+  <si>
+    <t>Em frente a 2A importados - R. Cândido Mendes, 1189 - Central, Macapá - AP, 68900-100</t>
+  </si>
+  <si>
+    <t>Av. Barão de Capanema - Centro, Capanema - PA, 68700-005</t>
+  </si>
+  <si>
+    <t>Rua Manoel Barata, 581, Cruzeiro, Icoaraci, Belém - PA, 66810100</t>
+  </si>
+  <si>
+    <t>Av. Sen. Lemos, 3153 - Sacramenta, Belém - PA, 66120-000</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1641,8 +1753,40 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1667,8 +1811,14 @@
         <bgColor rgb="FFD9D9D9"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF000000"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="4">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -1713,11 +1863,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
@@ -1730,6 +1891,18 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2419,6 +2592,358 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{40DD5561-C71A-4E3E-8C3F-36B212A5A12C}">
+  <dimension ref="A1:D24"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="27.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="59.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.21875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" s="21" t="s">
+        <v>552</v>
+      </c>
+      <c r="B1" s="22" t="s">
+        <v>467</v>
+      </c>
+      <c r="C1" s="23" t="s">
+        <v>553</v>
+      </c>
+      <c r="D1" s="23" t="s">
+        <v>554</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" s="12" t="s">
+        <v>414</v>
+      </c>
+      <c r="B2" s="13">
+        <v>1</v>
+      </c>
+      <c r="C2" s="14" t="s">
+        <v>525</v>
+      </c>
+      <c r="D2" s="14" t="s">
+        <v>526</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" s="15" t="s">
+        <v>415</v>
+      </c>
+      <c r="B3" s="16">
+        <v>2</v>
+      </c>
+      <c r="C3" s="17" t="s">
+        <v>527</v>
+      </c>
+      <c r="D3" s="17" t="s">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" s="12" t="s">
+        <v>416</v>
+      </c>
+      <c r="B4" s="13">
+        <v>3</v>
+      </c>
+      <c r="C4" s="14" t="s">
+        <v>529</v>
+      </c>
+      <c r="D4" s="14" t="s">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" s="15" t="s">
+        <v>417</v>
+      </c>
+      <c r="B5" s="16">
+        <v>4</v>
+      </c>
+      <c r="C5" s="17" t="s">
+        <v>531</v>
+      </c>
+      <c r="D5" s="18" t="s">
+        <v>532</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6" s="12" t="s">
+        <v>418</v>
+      </c>
+      <c r="B6" s="13">
+        <v>5</v>
+      </c>
+      <c r="C6" s="14" t="s">
+        <v>533</v>
+      </c>
+      <c r="D6" s="14" t="s">
+        <v>534</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7" s="15" t="s">
+        <v>419</v>
+      </c>
+      <c r="B7" s="16">
+        <v>6</v>
+      </c>
+      <c r="C7" s="17" t="s">
+        <v>535</v>
+      </c>
+      <c r="D7" s="18" t="s">
+        <v>534</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8" s="12" t="s">
+        <v>420</v>
+      </c>
+      <c r="B8" s="13">
+        <v>7</v>
+      </c>
+      <c r="C8" s="19" t="s">
+        <v>536</v>
+      </c>
+      <c r="D8" s="14" t="s">
+        <v>532</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A9" s="15" t="s">
+        <v>421</v>
+      </c>
+      <c r="B9" s="16">
+        <v>8</v>
+      </c>
+      <c r="C9" s="17" t="s">
+        <v>537</v>
+      </c>
+      <c r="D9" s="18" t="s">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A10" s="12" t="s">
+        <v>422</v>
+      </c>
+      <c r="B10" s="13">
+        <v>9</v>
+      </c>
+      <c r="C10" s="19" t="s">
+        <v>537</v>
+      </c>
+      <c r="D10" s="14" t="s">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A11" s="15" t="s">
+        <v>423</v>
+      </c>
+      <c r="B11" s="16">
+        <v>10</v>
+      </c>
+      <c r="C11" s="17" t="s">
+        <v>538</v>
+      </c>
+      <c r="D11" s="18" t="s">
+        <v>539</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A12" s="12" t="s">
+        <v>424</v>
+      </c>
+      <c r="B12" s="13">
+        <v>11</v>
+      </c>
+      <c r="C12" s="19" t="s">
+        <v>540</v>
+      </c>
+      <c r="D12" s="14" t="s">
+        <v>539</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A13" s="15" t="s">
+        <v>425</v>
+      </c>
+      <c r="B13" s="16">
+        <v>12</v>
+      </c>
+      <c r="C13" s="17" t="s">
+        <v>540</v>
+      </c>
+      <c r="D13" s="18" t="s">
+        <v>539</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A14" s="12" t="s">
+        <v>426</v>
+      </c>
+      <c r="B14" s="13">
+        <v>13</v>
+      </c>
+      <c r="C14" s="19" t="s">
+        <v>541</v>
+      </c>
+      <c r="D14" s="14" t="s">
+        <v>542</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A15" s="15" t="s">
+        <v>427</v>
+      </c>
+      <c r="B15" s="16">
+        <v>14</v>
+      </c>
+      <c r="C15" s="17" t="s">
+        <v>543</v>
+      </c>
+      <c r="D15" s="18" t="s">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A16" s="12" t="s">
+        <v>428</v>
+      </c>
+      <c r="B16" s="13">
+        <v>15</v>
+      </c>
+      <c r="C16" s="20" t="s">
+        <v>543</v>
+      </c>
+      <c r="D16" s="14" t="s">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A17" s="15" t="s">
+        <v>429</v>
+      </c>
+      <c r="B17" s="16">
+        <v>16</v>
+      </c>
+      <c r="C17" s="17" t="s">
+        <v>544</v>
+      </c>
+      <c r="D17" s="18" t="s">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A18" s="12" t="s">
+        <v>545</v>
+      </c>
+      <c r="B18" s="13">
+        <v>17</v>
+      </c>
+      <c r="C18" s="19" t="s">
+        <v>546</v>
+      </c>
+      <c r="D18" s="14" t="s">
+        <v>547</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A19" s="15" t="s">
+        <v>431</v>
+      </c>
+      <c r="B19" s="16">
+        <v>18</v>
+      </c>
+      <c r="C19" s="18" t="s">
+        <v>557</v>
+      </c>
+      <c r="D19" s="18" t="s">
+        <v>548</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A20" s="12" t="s">
+        <v>432</v>
+      </c>
+      <c r="B20" s="13">
+        <v>19</v>
+      </c>
+      <c r="C20" s="14" t="s">
+        <v>558</v>
+      </c>
+      <c r="D20" s="14" t="s">
+        <v>549</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A21" s="15" t="s">
+        <v>433</v>
+      </c>
+      <c r="B21" s="16">
+        <v>20</v>
+      </c>
+      <c r="C21" s="18" t="s">
+        <v>559</v>
+      </c>
+      <c r="D21" s="18" t="s">
+        <v>550</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A22" s="12" t="s">
+        <v>434</v>
+      </c>
+      <c r="B22" s="13">
+        <v>21</v>
+      </c>
+      <c r="C22" s="14" t="s">
+        <v>560</v>
+      </c>
+      <c r="D22" s="14" t="s">
+        <v>551</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A23" s="15" t="s">
+        <v>524</v>
+      </c>
+      <c r="B23" s="16">
+        <v>22</v>
+      </c>
+      <c r="C23" s="18" t="s">
+        <v>555</v>
+      </c>
+      <c r="D23" s="18" t="s">
+        <v>556</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A24" s="12" t="s">
+        <v>523</v>
+      </c>
+      <c r="B24" s="13">
+        <v>23</v>
+      </c>
+      <c r="C24" s="14" t="s">
+        <v>561</v>
+      </c>
+      <c r="D24" s="14" t="s">
+        <v>528</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F4489C6B-D1C2-415E-B0B3-CC749A9F03E5}">
   <dimension ref="A1:C234"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -5007,7 +5532,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{206F00A0-332C-413C-836F-690379DEF35A}">
   <dimension ref="A1:B7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -5080,7 +5605,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{525F9421-13B4-413F-B405-CE8C1993584F}">
   <dimension ref="A1:B6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>

</xml_diff>